<commit_message>
Count only reachable hosts into ccsp (#79)
* Only count hosts that are reachable

If host has all tasks in unreachable/dark state, we don't want
to count it into list of managed nodes.

Issue: https://issues.redhat.com/browse/AAP-38736

* Update snapshot tests

Removing unreachable hosts changes all reports
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-05--2024-04-30/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-05--2024-04-30/report.xlsx
@@ -733,7 +733,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr"/>
       <c r="C18" s="9" t="n">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="D18" s="10" t="n">
         <v>15.01</v>
@@ -822,7 +822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F275"/>
+  <dimension ref="A1:F266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6527,51 +6527,51 @@
     <row r="259">
       <c r="A259" s="12" t="inlineStr">
         <is>
-          <t>my_first_test 14</t>
+          <t>my_first_test 694</t>
         </is>
       </c>
       <c r="B259" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C259" s="12" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D259" s="12" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E259" s="13" t="n">
-        <v>45399.01062650024</v>
+        <v>45399.4408509534</v>
       </c>
       <c r="F259" s="13" t="n">
-        <v>45399.38562644433</v>
+        <v>45399.4408509534</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="12" t="inlineStr">
         <is>
-          <t>my_first_test 148</t>
+          <t>my_test</t>
         </is>
       </c>
       <c r="B260" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C260" s="12" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D260" s="12" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E260" s="13" t="n">
-        <v>45399.01062649558</v>
+        <v>45399.43640744589</v>
       </c>
       <c r="F260" s="13" t="n">
-        <v>45399.38562643925</v>
+        <v>45399.4408509517</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="12" t="inlineStr">
         <is>
-          <t>my_first_test 15</t>
+          <t>test host 1</t>
         </is>
       </c>
       <c r="B261" s="12" t="n">
@@ -6581,19 +6581,19 @@
         <v>10</v>
       </c>
       <c r="D261" s="12" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E261" s="13" t="n">
-        <v>45399.01062649627</v>
+        <v>45350.36714858868</v>
       </c>
       <c r="F261" s="13" t="n">
-        <v>45399.38562644007</v>
+        <v>45369.66744835266</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="12" t="inlineStr">
         <is>
-          <t>my_first_test 16</t>
+          <t>test host 2</t>
         </is>
       </c>
       <c r="B262" s="12" t="n">
@@ -6603,85 +6603,85 @@
         <v>10</v>
       </c>
       <c r="D262" s="12" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E262" s="13" t="n">
-        <v>45399.0106264992</v>
+        <v>45350.36714858697</v>
       </c>
       <c r="F262" s="13" t="n">
-        <v>45399.38562644357</v>
+        <v>45369.66744833602</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="12" t="inlineStr">
         <is>
-          <t>my_first_test 18</t>
+          <t>test_ansible_host_real_1</t>
         </is>
       </c>
       <c r="B263" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C263" s="12" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D263" s="12" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E263" s="13" t="n">
-        <v>45399.01062649854</v>
+        <v>45369.62322191329</v>
       </c>
       <c r="F263" s="13" t="n">
-        <v>45399.38562644275</v>
+        <v>45369.66744835195</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="12" t="inlineStr">
         <is>
-          <t>my_first_test 26</t>
+          <t>test_ansible_host_real_2</t>
         </is>
       </c>
       <c r="B264" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C264" s="12" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D264" s="12" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E264" s="13" t="n">
-        <v>45399.01062649232</v>
+        <v>45369.62322191397</v>
       </c>
       <c r="F264" s="13" t="n">
-        <v>45399.38562643561</v>
+        <v>45369.66744835246</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="12" t="inlineStr">
         <is>
-          <t>my_first_test 338</t>
+          <t>test_host_3</t>
         </is>
       </c>
       <c r="B265" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C265" s="12" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D265" s="12" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E265" s="13" t="n">
-        <v>45399.01062649694</v>
+        <v>45362.32864392176</v>
       </c>
       <c r="F265" s="13" t="n">
-        <v>45399.38562644089</v>
+        <v>45369.66744835159</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="12" t="inlineStr">
         <is>
-          <t>my_first_test 694</t>
+          <t>test_json_host_1</t>
         </is>
       </c>
       <c r="B266" s="12" t="n">
@@ -6694,207 +6694,9 @@
         <v>2</v>
       </c>
       <c r="E266" s="13" t="n">
-        <v>45399.4408509534</v>
+        <v>45369.66744835285</v>
       </c>
       <c r="F266" s="13" t="n">
-        <v>45399.4408509534</v>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" s="12" t="inlineStr">
-        <is>
-          <t>my_first_test 7</t>
-        </is>
-      </c>
-      <c r="B267" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C267" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="D267" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="E267" s="13" t="n">
-        <v>45399.01062649394</v>
-      </c>
-      <c r="F267" s="13" t="n">
-        <v>45399.3856264374</v>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" s="12" t="inlineStr">
-        <is>
-          <t>my_first_test 78</t>
-        </is>
-      </c>
-      <c r="B268" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C268" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="D268" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="E268" s="13" t="n">
-        <v>45399.01062649785</v>
-      </c>
-      <c r="F268" s="13" t="n">
-        <v>45399.38562644191</v>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" s="12" t="inlineStr">
-        <is>
-          <t>my_test</t>
-        </is>
-      </c>
-      <c r="B269" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C269" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="D269" s="12" t="n">
-        <v>11</v>
-      </c>
-      <c r="E269" s="13" t="n">
-        <v>45399.4256597221</v>
-      </c>
-      <c r="F269" s="13" t="n">
-        <v>45399.4408509517</v>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" s="12" t="inlineStr">
-        <is>
-          <t>test host 1</t>
-        </is>
-      </c>
-      <c r="B270" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C270" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="D270" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="E270" s="13" t="n">
-        <v>45350.36714858868</v>
-      </c>
-      <c r="F270" s="13" t="n">
-        <v>45369.66744835266</v>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" s="12" t="inlineStr">
-        <is>
-          <t>test host 2</t>
-        </is>
-      </c>
-      <c r="B271" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C271" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="D271" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="E271" s="13" t="n">
-        <v>45350.36714858697</v>
-      </c>
-      <c r="F271" s="13" t="n">
-        <v>45369.66744833602</v>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" s="12" t="inlineStr">
-        <is>
-          <t>test_ansible_host_real_1</t>
-        </is>
-      </c>
-      <c r="B272" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C272" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D272" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E272" s="13" t="n">
-        <v>45369.62322191329</v>
-      </c>
-      <c r="F272" s="13" t="n">
-        <v>45369.66744835195</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" s="12" t="inlineStr">
-        <is>
-          <t>test_ansible_host_real_2</t>
-        </is>
-      </c>
-      <c r="B273" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C273" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D273" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="E273" s="13" t="n">
-        <v>45369.62322191397</v>
-      </c>
-      <c r="F273" s="13" t="n">
-        <v>45369.66744835246</v>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" s="12" t="inlineStr">
-        <is>
-          <t>test_host_3</t>
-        </is>
-      </c>
-      <c r="B274" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C274" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D274" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="E274" s="13" t="n">
-        <v>45362.32864392176</v>
-      </c>
-      <c r="F274" s="13" t="n">
-        <v>45369.66744835159</v>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" s="12" t="inlineStr">
-        <is>
-          <t>test_json_host_1</t>
-        </is>
-      </c>
-      <c r="B275" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C275" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D275" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E275" s="13" t="n">
-        <v>45369.66744835285</v>
-      </c>
-      <c r="F275" s="13" t="n">
         <v>45369.66744835285</v>
       </c>
     </row>

</xml_diff>